<commit_message>
update đơn hàng sản phẩm be
</commit_message>
<xml_diff>
--- a/phong-tap-be/phong_tap-be/QuanLyPhongGym/src/main/resources/template/doanh-thu-template.xlsx
+++ b/phong-tap-be/phong_tap-be/QuanLyPhongGym/src/main/resources/template/doanh-thu-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Angular\DuAnDemo\quan-ly-phong-gym\phong-tap-be\phong_tap-be\QuanLyPhongGym\src\main\resources\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E8BD15-53FA-4E71-A899-526E2683FC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB7CB15-6FB2-496B-ACEE-B79E1EB311E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1995" windowWidth="29040" windowHeight="15720" xr2:uid="{512CA105-0148-4CEB-AD2C-388E7B3175FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{512CA105-0148-4CEB-AD2C-388E7B3175FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="_([$VND]\ * #,##0_);_([$VND]\ * \(#,##0\);_([$VND]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_([$VND]\ * #,##0_);_([$VND]\ * \(#,##0\);_([$VND]\ * &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -155,17 +155,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -482,26 +482,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F760B8C-5FBD-4737-A224-1FB3BA035C32}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="17" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="27" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="6" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:6" ht="29.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="29.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -519,7 +519,7 @@
       </c>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -532,19 +532,19 @@
       <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" ht="29.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:6" ht="29.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="6"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:E3" xr:uid="{7F760B8C-5FBD-4737-A224-1FB3BA035C32}"/>

</xml_diff>